<commit_message>
Migración a datos de validación reales, des-transformación de predicciones y visualización proporcional con paleta jet
</commit_message>
<xml_diff>
--- a/data/processed/tabla_resultados_modelos_tesina.xlsx
+++ b/data/processed/tabla_resultados_modelos_tesina.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados modelos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,11 +26,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
-    </font>
-    <font>
       <b val="1"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,17 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,125 +425,75 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tabla 2: Resultados de modelos de predicción (validación). Número de datos de evaluación por modelo según partición train/test. (Letra 10, espaciado simple.)</t>
-        </is>
+          <t>Modelo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>R2 (unidades reales)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>RMSE (unidades reales)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Sesgo (Bias %)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>343732</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.1482120666961944</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.852709109509887</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.01599757706585076</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Modelo</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>R²</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>RMSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>(1)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>(2)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>(3)</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>(4)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>KNN</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>248</v>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>0.3929</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>0.8011</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>248</v>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>0.4285</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>0.7772</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Nota:</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>(a) Elaboración propia. N = número de datos en conjunto de evaluación (test). R² = coeficiente de determinación. RMSE = raíz del error cuadrático medio. Si se reporta ±, corresponde a desviación estándar sobre múltiples particiones.</t>
-        </is>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>XGB</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>343732</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-0.1446155492489301</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.466119082902512</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.08148808062571765</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: standardizar scripts visualización ML y validación por UE
</commit_message>
<xml_diff>
--- a/data/processed/tabla_resultados_modelos_tesina.xlsx
+++ b/data/processed/tabla_resultados_modelos_tesina.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,13 +465,13 @@
         <v>343732</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1482120666961944</v>
+        <v>0.2535669010937576</v>
       </c>
       <c r="D2" t="n">
-        <v>3.852709109509887</v>
+        <v>3.606582927705258</v>
       </c>
       <c r="E2" t="n">
-        <v>0.01599757706585076</v>
+        <v>-0.3171831563159282</v>
       </c>
     </row>
     <row r="3">
@@ -484,13 +484,51 @@
         <v>343732</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.1446155492489301</v>
+        <v>-0.1399380700703119</v>
       </c>
       <c r="D3" t="n">
-        <v>4.466119082902512</v>
+        <v>4.456984328129871</v>
       </c>
       <c r="E3" t="n">
-        <v>0.08148808062571765</v>
+        <v>0.06571810635271479</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SVR</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>343732</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.2209819924688748</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3.684463227762158</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-0.7459061018770916</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>343732</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.2176870888490069</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3.692246835792068</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-0.4245929972879214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Añadido 06.validacion_espacial.py con comparativas visuales y estadisticas de Machine Learning emparejadas
</commit_message>
<xml_diff>
--- a/data/processed/tabla_resultados_modelos_tesina.xlsx
+++ b/data/processed/tabla_resultados_modelos_tesina.xlsx
@@ -465,10 +465,10 @@
         <v>343732</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2535669010937577</v>
+        <v>0.2535669010937576</v>
       </c>
       <c r="D2" t="n">
-        <v>3.606582927705257</v>
+        <v>3.606582927705258</v>
       </c>
       <c r="E2" t="n">
         <v>-0.3171831563159281</v>
@@ -484,13 +484,13 @@
         <v>343732</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.1399380700703117</v>
+        <v>-0.1399380700703119</v>
       </c>
       <c r="D3" t="n">
-        <v>4.45698432812987</v>
+        <v>4.456984328129871</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06571810635271473</v>
+        <v>0.06571810635271479</v>
       </c>
     </row>
     <row r="4">
@@ -503,13 +503,13 @@
         <v>343732</v>
       </c>
       <c r="C4" t="n">
-        <v>0.2209819924688748</v>
+        <v>0.220981992468875</v>
       </c>
       <c r="D4" t="n">
         <v>3.684463227762158</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.7459061018770908</v>
+        <v>-0.7459061018770912</v>
       </c>
     </row>
     <row r="5">
@@ -528,7 +528,7 @@
         <v>3.692246835792068</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.4245929972879212</v>
+        <v>-0.424592997287921</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualización de scripts, datos y resultados de validación espacial
</commit_message>
<xml_diff>
--- a/data/processed/tabla_resultados_modelos_tesina.xlsx
+++ b/data/processed/tabla_resultados_modelos_tesina.xlsx
@@ -465,13 +465,13 @@
         <v>343732</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2535669010937576</v>
+        <v>0.1841831040982762</v>
       </c>
       <c r="D2" t="n">
-        <v>3.606582927705258</v>
+        <v>3.770481600409159</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.3171831563159281</v>
+        <v>-0.3669280272116155</v>
       </c>
     </row>
     <row r="3">
@@ -484,13 +484,13 @@
         <v>343732</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.1399380700703119</v>
+        <v>0.05953485243518486</v>
       </c>
       <c r="D3" t="n">
-        <v>4.456984328129871</v>
+        <v>4.048292006464415</v>
       </c>
       <c r="E3" t="n">
-        <v>0.06571810635271479</v>
+        <v>-0.1758181423902269</v>
       </c>
     </row>
     <row r="4">
@@ -503,13 +503,13 @@
         <v>343732</v>
       </c>
       <c r="C4" t="n">
-        <v>0.220981992468875</v>
+        <v>0.08073480876334893</v>
       </c>
       <c r="D4" t="n">
-        <v>3.684463227762158</v>
+        <v>4.002403648940446</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.7459061018770912</v>
+        <v>-0.3628528064045478</v>
       </c>
     </row>
     <row r="5">
@@ -522,13 +522,13 @@
         <v>343732</v>
       </c>
       <c r="C5" t="n">
-        <v>0.2176870888490069</v>
+        <v>0.07894261911106293</v>
       </c>
       <c r="D5" t="n">
-        <v>3.692246835792068</v>
+        <v>4.00630327102045</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.424592997287921</v>
+        <v>-0.468601770461472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>